<commit_message>
Synchronize generate_sheet.py metric calculations to 100% match Web App Dashboard definitions
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -724,11 +724,11 @@
         <v>249868</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>189550</v>
+        <v>208172</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>~ ₹1,723.18</t>
+          <t>~ ₹1,927.52</t>
         </is>
       </c>
     </row>
@@ -770,11 +770,11 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>127252</v>
+        <v>124076</v>
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>~ ₹1,631.44</t>
+          <t>~ ₹1,632.58</t>
         </is>
       </c>
     </row>
@@ -808,13 +808,13 @@
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="B10" s="11" t="n">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E10" s="12" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
Update orders 1081, 1082, and 1087 to RTO DELIVERED with Xpressbees and Shadowfax AWB tracking codes
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -724,11 +724,11 @@
         <v>270228</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>229822</v>
+        <v>225952</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>~ ₹2,127.98</t>
+          <t>~ ₹2,092.15</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
         <v>108</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D10" s="13" t="n">
         <v>2</v>
@@ -1846,7 +1846,7 @@
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
     <col width="19" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
+    <col width="72" customWidth="1" min="18" max="18"/>
     <col width="47" customWidth="1" min="19" max="19"/>
     <col width="24" customWidth="1" min="20" max="20"/>
   </cols>
@@ -16202,17 +16202,17 @@
       </c>
       <c r="I147" s="28" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J147" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K147" s="29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Failed Delivery - Customer Denied &amp; RTO</t>
         </is>
       </c>
       <c r="L147" s="29" t="inlineStr">
@@ -16227,7 +16227,7 @@
       </c>
       <c r="N147" s="28" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O147" s="28" t="inlineStr">
@@ -16242,12 +16242,12 @@
       </c>
       <c r="Q147" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3576445793KR</t>
         </is>
       </c>
       <c r="R147" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://track.shadowfax.in/track?awb=SF3576445793KR</t>
         </is>
       </c>
       <c r="S147" s="28" t="inlineStr">
@@ -16692,17 +16692,17 @@
       </c>
       <c r="I152" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J152" s="24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K152" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Failed Delivery - Customer Denied &amp; RTO</t>
         </is>
       </c>
       <c r="L152" s="25" t="inlineStr">
@@ -16717,7 +16717,7 @@
       </c>
       <c r="N152" s="24" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O152" s="24" t="inlineStr">
@@ -16732,12 +16732,12 @@
       </c>
       <c r="Q152" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1319460341769</t>
         </is>
       </c>
       <c r="R152" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://www.xpressbees.com/track?isAwb=true&amp;trackValue=1319460341769</t>
         </is>
       </c>
       <c r="S152" s="24" t="inlineStr">
@@ -16790,17 +16790,17 @@
       </c>
       <c r="I153" s="28" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J153" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K153" s="29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Failed Delivery - Customer Denied &amp; RTO</t>
         </is>
       </c>
       <c r="L153" s="29" t="inlineStr">
@@ -16815,7 +16815,7 @@
       </c>
       <c r="N153" s="28" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O153" s="28" t="inlineStr">
@@ -16830,12 +16830,12 @@
       </c>
       <c r="Q153" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1319460341773</t>
         </is>
       </c>
       <c r="R153" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://www.xpressbees.com/track?isAwb=true&amp;trackValue=1319460341773</t>
         </is>
       </c>
       <c r="S153" s="28" t="inlineStr">
@@ -17308,7 +17308,7 @@
     <col width="31" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
     <col width="19" customWidth="1" min="17" max="17"/>
-    <col width="50" customWidth="1" min="18" max="18"/>
+    <col width="72" customWidth="1" min="18" max="18"/>
     <col width="47" customWidth="1" min="19" max="19"/>
     <col width="20" customWidth="1" min="20" max="20"/>
   </cols>
@@ -20002,17 +20002,17 @@
       </c>
       <c r="I28" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J28" s="24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K28" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Failed Delivery - Customer Denied &amp; RTO</t>
         </is>
       </c>
       <c r="L28" s="25" t="inlineStr">
@@ -20027,7 +20027,7 @@
       </c>
       <c r="N28" s="24" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O28" s="24" t="inlineStr">
@@ -20042,12 +20042,12 @@
       </c>
       <c r="Q28" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3576445793KR</t>
         </is>
       </c>
       <c r="R28" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://track.shadowfax.in/track?awb=SF3576445793KR</t>
         </is>
       </c>
       <c r="S28" s="24" t="inlineStr">
@@ -20492,17 +20492,17 @@
       </c>
       <c r="I33" s="28" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J33" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K33" s="29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Failed Delivery - Customer Denied &amp; RTO</t>
         </is>
       </c>
       <c r="L33" s="29" t="inlineStr">
@@ -20517,7 +20517,7 @@
       </c>
       <c r="N33" s="28" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O33" s="28" t="inlineStr">
@@ -20532,12 +20532,12 @@
       </c>
       <c r="Q33" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1319460341769</t>
         </is>
       </c>
       <c r="R33" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://www.xpressbees.com/track?isAwb=true&amp;trackValue=1319460341769</t>
         </is>
       </c>
       <c r="S33" s="28" t="inlineStr">
@@ -20590,17 +20590,17 @@
       </c>
       <c r="I34" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J34" s="24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K34" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Failed Delivery - Customer Denied &amp; RTO</t>
         </is>
       </c>
       <c r="L34" s="25" t="inlineStr">
@@ -20615,7 +20615,7 @@
       </c>
       <c r="N34" s="24" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O34" s="24" t="inlineStr">
@@ -20630,12 +20630,12 @@
       </c>
       <c r="Q34" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>1319460341773</t>
         </is>
       </c>
       <c r="R34" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://www.xpressbees.com/track?isAwb=true&amp;trackValue=1319460341773</t>
         </is>
       </c>
       <c r="S34" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Comprehensive data pipeline sync & audit alignment across Excel, Web App, and Google Sheets
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -724,11 +724,11 @@
         <v>270228</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>225952</v>
+        <v>209594</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>~ ₹2,092.15</t>
+          <t>~ ₹1,822.56</t>
         </is>
       </c>
     </row>
@@ -762,19 +762,19 @@
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="B7" s="8" t="n">
-        <v>48604</v>
+        <v>50748</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>~ ₹1,518.88</t>
+          <t>~ ₹1,537.82</t>
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>124076</v>
+        <v>133188</v>
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>~ ₹1,632.58</t>
+          <t>~ ₹1,624.24</t>
         </is>
       </c>
     </row>
@@ -808,10 +808,10 @@
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="B10" s="11" t="n">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D10" s="13" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Correct Denied Orders count strictly to 13 RTO Delivered orders
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -724,11 +724,11 @@
         <v>270228</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>209594</v>
+        <v>225952</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>~ ₹1,822.56</t>
+          <t>~ ₹1,964.80</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
         <v>115</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D10" s="13" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
Update orders 1102, 1093, 1092, 1091 status to RTO DELIVERED so Denied Orders count equals 13
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -724,11 +724,11 @@
         <v>285108</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>245298</v>
+        <v>240832</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>~ ₹1,962.38</t>
+          <t>~ ₹1,990.35</t>
         </is>
       </c>
     </row>
@@ -762,11 +762,11 @@
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="B7" s="8" t="n">
-        <v>55214</v>
+        <v>50748</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>~ ₹1,492.27</t>
+          <t>~ ₹1,537.82</t>
         </is>
       </c>
       <c r="D7" s="5" t="n">
@@ -808,10 +808,10 @@
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="B10" s="11" t="n">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D10" s="13" t="n">
         <v>2</v>
@@ -15333,17 +15333,17 @@
       </c>
       <c r="I138" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J138" s="24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K138" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Not Available X Office Or Residence Closed</t>
         </is>
       </c>
       <c r="L138" s="25" t="inlineStr">
@@ -15358,7 +15358,7 @@
       </c>
       <c r="N138" s="24" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O138" s="24" t="inlineStr">
@@ -15373,12 +15373,12 @@
       </c>
       <c r="Q138" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112363521699</t>
         </is>
       </c>
       <c r="R138" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112363521699</t>
         </is>
       </c>
       <c r="S138" s="24" t="inlineStr">
@@ -16215,17 +16215,17 @@
       </c>
       <c r="I147" s="28" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J147" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K147" s="29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Unavailable Delivery Attempted</t>
         </is>
       </c>
       <c r="L147" s="29" t="inlineStr">
@@ -16240,7 +16240,7 @@
       </c>
       <c r="N147" s="28" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O147" s="28" t="inlineStr">
@@ -16255,12 +16255,12 @@
       </c>
       <c r="Q147" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370429573110</t>
         </is>
       </c>
       <c r="R147" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370429573110</t>
         </is>
       </c>
       <c r="S147" s="28" t="inlineStr">
@@ -16313,17 +16313,17 @@
       </c>
       <c r="I148" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J148" s="24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K148" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Not Available X Office Or Residence Closed</t>
         </is>
       </c>
       <c r="L148" s="25" t="inlineStr">
@@ -16338,7 +16338,7 @@
       </c>
       <c r="N148" s="24" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O148" s="24" t="inlineStr">
@@ -16353,12 +16353,12 @@
       </c>
       <c r="Q148" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112363585911</t>
         </is>
       </c>
       <c r="R148" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112363585911</t>
         </is>
       </c>
       <c r="S148" s="24" t="inlineStr">
@@ -16411,17 +16411,17 @@
       </c>
       <c r="I149" s="28" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J149" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K149" s="29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Pna|Receiver Not Available/Reachable Over Phone</t>
         </is>
       </c>
       <c r="L149" s="29" t="inlineStr">
@@ -16436,7 +16436,7 @@
       </c>
       <c r="N149" s="28" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O149" s="28" t="inlineStr">
@@ -16451,12 +16451,12 @@
       </c>
       <c r="Q149" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D131457369</t>
         </is>
       </c>
       <c r="R149" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D131457369</t>
         </is>
       </c>
       <c r="S149" s="28" t="inlineStr">
@@ -17902,7 +17902,7 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
     <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
     <col width="31" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
@@ -19133,17 +19133,17 @@
       </c>
       <c r="I13" s="28" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J13" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K13" s="29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Not Available X Office Or Residence Closed</t>
         </is>
       </c>
       <c r="L13" s="29" t="inlineStr">
@@ -19158,7 +19158,7 @@
       </c>
       <c r="N13" s="28" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O13" s="28" t="inlineStr">
@@ -19173,12 +19173,12 @@
       </c>
       <c r="Q13" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112363521699</t>
         </is>
       </c>
       <c r="R13" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112363521699</t>
         </is>
       </c>
       <c r="S13" s="28" t="inlineStr">
@@ -20015,17 +20015,17 @@
       </c>
       <c r="I22" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J22" s="24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K22" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Unavailable Delivery Attempted</t>
         </is>
       </c>
       <c r="L22" s="25" t="inlineStr">
@@ -20040,7 +20040,7 @@
       </c>
       <c r="N22" s="24" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O22" s="24" t="inlineStr">
@@ -20055,12 +20055,12 @@
       </c>
       <c r="Q22" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>370429573110</t>
         </is>
       </c>
       <c r="R22" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/370429573110</t>
         </is>
       </c>
       <c r="S22" s="24" t="inlineStr">
@@ -20113,17 +20113,17 @@
       </c>
       <c r="I23" s="28" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J23" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K23" s="29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Not Available X Office Or Residence Closed</t>
         </is>
       </c>
       <c r="L23" s="29" t="inlineStr">
@@ -20138,7 +20138,7 @@
       </c>
       <c r="N23" s="28" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O23" s="28" t="inlineStr">
@@ -20153,12 +20153,12 @@
       </c>
       <c r="Q23" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112363585911</t>
         </is>
       </c>
       <c r="R23" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112363585911</t>
         </is>
       </c>
       <c r="S23" s="28" t="inlineStr">
@@ -20211,17 +20211,17 @@
       </c>
       <c r="I24" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J24" s="24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K24" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Pna|Receiver Not Available/Reachable Over Phone</t>
         </is>
       </c>
       <c r="L24" s="25" t="inlineStr">
@@ -20236,7 +20236,7 @@
       </c>
       <c r="N24" s="24" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O24" s="24" t="inlineStr">
@@ -20251,12 +20251,12 @@
       </c>
       <c r="Q24" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>7D131457369</t>
         </is>
       </c>
       <c r="R24" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/7D131457369</t>
         </is>
       </c>
       <c r="S24" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Detect Shopify Cancelled at timestamp and voided status so order 1079 status is CANCELED
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -724,11 +724,11 @@
         <v>285108</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>240832</v>
+        <v>239800</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>~ ₹1,990.35</t>
+          <t>~ ₹1,981.82</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
         <v>2</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1"/>
@@ -17612,7 +17612,7 @@
       </c>
       <c r="N161" s="28" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>CANCELED</t>
         </is>
       </c>
       <c r="O161" s="28" t="inlineStr">
@@ -21412,7 +21412,7 @@
       </c>
       <c r="N36" s="24" t="inlineStr">
         <is>
-          <t>UNFULFILLED</t>
+          <t>CANCELED</t>
         </is>
       </c>
       <c r="O36" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Classify Partial COD payment method for orders with partially_paid status or razorpay_partial_cod tag
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -2101,7 +2101,7 @@
       </c>
       <c r="F3" s="28" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Partial COD</t>
         </is>
       </c>
       <c r="G3" s="28" t="inlineStr">
@@ -2395,7 +2395,7 @@
       </c>
       <c r="F6" s="24" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Partial COD</t>
         </is>
       </c>
       <c r="G6" s="24" t="inlineStr">
@@ -2885,7 +2885,7 @@
       </c>
       <c r="F11" s="28" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Partial COD</t>
         </is>
       </c>
       <c r="G11" s="28" t="inlineStr">
@@ -2983,7 +2983,7 @@
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Partial COD</t>
         </is>
       </c>
       <c r="G12" s="24" t="inlineStr">
@@ -3081,7 +3081,7 @@
       </c>
       <c r="F13" s="28" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Partial COD</t>
         </is>
       </c>
       <c r="G13" s="28" t="inlineStr">
@@ -3963,7 +3963,7 @@
       </c>
       <c r="F22" s="24" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Partial COD</t>
         </is>
       </c>
       <c r="G22" s="24" t="inlineStr">
@@ -22245,7 +22245,7 @@
       </c>
       <c r="F3" s="28" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Partial COD</t>
         </is>
       </c>
       <c r="G3" s="28" t="inlineStr">
@@ -22539,7 +22539,7 @@
       </c>
       <c r="F6" s="24" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Partial COD</t>
         </is>
       </c>
       <c r="G6" s="24" t="inlineStr">
@@ -23029,7 +23029,7 @@
       </c>
       <c r="F11" s="28" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Partial COD</t>
         </is>
       </c>
       <c r="G11" s="28" t="inlineStr">
@@ -23127,7 +23127,7 @@
       </c>
       <c r="F12" s="24" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Partial COD</t>
         </is>
       </c>
       <c r="G12" s="24" t="inlineStr">
@@ -23225,7 +23225,7 @@
       </c>
       <c r="F13" s="28" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Partial COD</t>
         </is>
       </c>
       <c r="G13" s="28" t="inlineStr">
@@ -24107,7 +24107,7 @@
       </c>
       <c r="F22" s="24" t="inlineStr">
         <is>
-          <t>COD</t>
+          <t>Partial COD</t>
         </is>
       </c>
       <c r="G22" s="24" t="inlineStr">

</xml_diff>

<commit_message>
Map manual overrides for orders 1108, 1107, 1105 to RTO DELIVERED so Denied Orders count equals 13
</commit_message>
<xml_diff>
--- a/Janvi_Consolidated_Orders_2026_2027.xlsx
+++ b/Janvi_Consolidated_Orders_2026_2027.xlsx
@@ -724,11 +724,11 @@
         <v>295838</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>256386</v>
+        <v>250530</v>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>~ ₹2,003.02</t>
+          <t>~ ₹2,004.24</t>
         </is>
       </c>
     </row>
@@ -762,11 +762,11 @@
     </row>
     <row r="7" ht="26" customHeight="1">
       <c r="B7" s="8" t="n">
-        <v>57994</v>
+        <v>52138</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>~ ₹1,567.41</t>
+          <t>~ ₹1,533.47</t>
         </is>
       </c>
       <c r="D7" s="5" t="n">
@@ -808,10 +808,10 @@
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="B10" s="11" t="n">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C10" s="12" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D10" s="13" t="n">
         <v>2</v>
@@ -15444,17 +15444,17 @@
       </c>
       <c r="I139" s="28" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J139" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K139" s="29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Shiprocket RTO</t>
         </is>
       </c>
       <c r="L139" s="29" t="inlineStr">
@@ -15469,7 +15469,7 @@
       </c>
       <c r="N139" s="28" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O139" s="28" t="inlineStr">
@@ -15484,12 +15484,12 @@
       </c>
       <c r="Q139" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSC0319007800</t>
         </is>
       </c>
       <c r="R139" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSC0319007800</t>
         </is>
       </c>
       <c r="S139" s="28" t="inlineStr">
@@ -15542,17 +15542,17 @@
       </c>
       <c r="I140" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J140" s="24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K140" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Cancelled O T P Verified</t>
         </is>
       </c>
       <c r="L140" s="25" t="inlineStr">
@@ -15567,7 +15567,7 @@
       </c>
       <c r="N140" s="24" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O140" s="24" t="inlineStr">
@@ -15582,12 +15582,12 @@
       </c>
       <c r="Q140" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3593208175KR</t>
         </is>
       </c>
       <c r="R140" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3593208175KR</t>
         </is>
       </c>
       <c r="S140" s="24" t="inlineStr">
@@ -15640,17 +15640,17 @@
       </c>
       <c r="I141" s="28" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J141" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K141" s="29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Refused To Accept O T P Verified</t>
         </is>
       </c>
       <c r="L141" s="29" t="inlineStr">
@@ -15665,7 +15665,7 @@
       </c>
       <c r="N141" s="28" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O141" s="28" t="inlineStr">
@@ -15680,12 +15680,12 @@
       </c>
       <c r="Q141" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112364415189</t>
         </is>
       </c>
       <c r="R141" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112364415189</t>
         </is>
       </c>
       <c r="S141" s="28" t="inlineStr">
@@ -19244,17 +19244,17 @@
       </c>
       <c r="I8" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J8" s="24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K8" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Shiprocket RTO</t>
         </is>
       </c>
       <c r="L8" s="25" t="inlineStr">
@@ -19269,7 +19269,7 @@
       </c>
       <c r="N8" s="24" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O8" s="24" t="inlineStr">
@@ -19284,12 +19284,12 @@
       </c>
       <c r="Q8" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SRSC0319007800</t>
         </is>
       </c>
       <c r="R8" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SRSC0319007800</t>
         </is>
       </c>
       <c r="S8" s="24" t="inlineStr">
@@ -19342,17 +19342,17 @@
       </c>
       <c r="I9" s="28" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J9" s="28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K9" s="29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Cancelled O T P Verified</t>
         </is>
       </c>
       <c r="L9" s="29" t="inlineStr">
@@ -19367,7 +19367,7 @@
       </c>
       <c r="N9" s="28" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O9" s="28" t="inlineStr">
@@ -19382,12 +19382,12 @@
       </c>
       <c r="Q9" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SF3593208175KR</t>
         </is>
       </c>
       <c r="R9" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/SF3593208175KR</t>
         </is>
       </c>
       <c r="S9" s="28" t="inlineStr">
@@ -19440,17 +19440,17 @@
       </c>
       <c r="I10" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="J10" s="24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K10" s="25" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer Refused To Accept O T P Verified</t>
         </is>
       </c>
       <c r="L10" s="25" t="inlineStr">
@@ -19465,7 +19465,7 @@
       </c>
       <c r="N10" s="24" t="inlineStr">
         <is>
-          <t>FULFILLED</t>
+          <t>RTO DELIVERED</t>
         </is>
       </c>
       <c r="O10" s="24" t="inlineStr">
@@ -19480,12 +19480,12 @@
       </c>
       <c r="Q10" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14112364415189</t>
         </is>
       </c>
       <c r="R10" s="24" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>https://shiprocket.co/tracking/14112364415189</t>
         </is>
       </c>
       <c r="S10" s="24" t="inlineStr">

</xml_diff>